<commit_message>
update template and code
</commit_message>
<xml_diff>
--- a/services/ami/ami/ami_weekly_status_report/per_project/Sweetfoot2/Sweetfoot2_wsr_template.xlsx
+++ b/services/ami/ami/ami_weekly_status_report/per_project/Sweetfoot2/Sweetfoot2_wsr_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="1" state="visible" r:id="rId2"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="80">
   <si>
     <t xml:space="preserve">Vendor  RVX</t>
   </si>
@@ -305,6 +305,9 @@
     <t xml:space="preserve">{id}</t>
   </si>
   <si>
+    <t xml:space="preserve">{sg_sequence}</t>
+  </si>
+  <si>
     <t xml:space="preserve">{sg_client_shot_name}</t>
   </si>
   <si>
@@ -314,7 +317,7 @@
     <t xml:space="preserve">{sg_next_delivery}</t>
   </si>
   <si>
-    <t xml:space="preserve">Test Description</t>
+    <t xml:space="preserve">{sg_vfx_work}</t>
   </si>
   <si>
     <t xml:space="preserve">{sg_status_list}</t>
@@ -361,7 +364,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">mm/dd/yyyy</t>
+    <t xml:space="preserve">{sg_pot_final_comp}</t>
   </si>
   <si>
     <t xml:space="preserve">{sg_notes}</t>
@@ -519,10 +522,16 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Description</t>
+    <t xml:space="preserve">[[asset]]</t>
   </si>
   <si>
     <t xml:space="preserve">{modeling___sg_blocking_date}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{texturing___sg_blocking_date}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mm/dd/yyyy</t>
   </si>
   <si>
     <t xml:space="preserve">{lookdev___sg_final_date}</t>
@@ -536,7 +545,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -616,6 +625,12 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -803,7 +818,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -966,6 +981,10 @@
     </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -2483,17 +2502,20 @@
   <dimension ref="A1:W1048576"/>
   <sheetFormatPr defaultColWidth="11.20703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="35.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="11" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="32.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="26.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="25.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="25.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="18.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="15" style="0" width="10.56"/>
   </cols>
   <sheetData>
@@ -2571,41 +2593,41 @@
       <c r="B3" s="33" t="n">
         <v>201</v>
       </c>
-      <c r="C3" s="33" t="n">
-        <v>1001</v>
+      <c r="C3" s="31" t="s">
+        <v>53</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>55</v>
-      </c>
-      <c r="G3" s="33" t="s">
         <v>56</v>
       </c>
+      <c r="G3" s="31" t="s">
+        <v>57</v>
+      </c>
       <c r="H3" s="31" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I3" s="33" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J3" s="31" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K3" s="31" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L3" s="34" t="s">
-        <v>61</v>
-      </c>
-      <c r="M3" s="33" t="s">
         <v>62</v>
       </c>
+      <c r="M3" s="31" t="s">
+        <v>63</v>
+      </c>
       <c r="N3" s="31" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O3" s="31"/>
       <c r="P3" s="31"/>
@@ -2616,7 +2638,7 @@
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4" s="31"/>
       <c r="C4" s="31"/>
@@ -3877,113 +3899,111 @@
   <dimension ref="A1:M1048576"/>
   <sheetFormatPr defaultColWidth="11.20703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="18.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="20.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="19.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="35.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="21.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.97"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="27.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="23.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="10.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="10.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="14" style="0" width="10.56"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="40.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="49.95" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C1" s="24" t="s">
         <v>38</v>
       </c>
       <c r="D1" s="26" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F1" s="40" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G1" s="28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H1" s="29" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I1" s="29" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J1" s="29" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K1" s="29" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="33" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="33" t="n">
-        <v>101</v>
-      </c>
-      <c r="D2" s="33" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" s="31" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="31" t="s">
-        <v>55</v>
-      </c>
-      <c r="G2" s="31" t="s">
+      <c r="A2" s="41" t="s">
         <v>75</v>
-      </c>
-      <c r="H2" s="33" t="s">
-        <v>62</v>
-      </c>
-      <c r="I2" s="33" t="s">
-        <v>62</v>
-      </c>
-      <c r="J2" s="31" t="s">
-        <v>76</v>
-      </c>
-      <c r="K2" s="31" t="s">
-        <v>63</v>
       </c>
       <c r="L2" s="35"/>
       <c r="M2" s="31"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="41"/>
-      <c r="H3" s="41"/>
-      <c r="I3" s="41"/>
-      <c r="J3" s="41"/>
+      <c r="A3" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="33" t="n">
+        <v>101</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="E3" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="F3" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="H3" s="31" t="s">
+        <v>77</v>
+      </c>
+      <c r="I3" s="33" t="s">
+        <v>78</v>
+      </c>
+      <c r="J3" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="K3" s="31" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="41" t="s">
+        <v>65</v>
+      </c>
       <c r="B4" s="32"/>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
       <c r="E4" s="32"/>
       <c r="F4" s="32"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
+      <c r="G4" s="42"/>
+      <c r="H4" s="42"/>
+      <c r="I4" s="42"/>
+      <c r="J4" s="42"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="32"/>
@@ -3991,10 +4011,10 @@
       <c r="D5" s="32"/>
       <c r="E5" s="32"/>
       <c r="F5" s="32"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
-      <c r="I5" s="41"/>
-      <c r="J5" s="41"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="32"/>
@@ -4002,10 +4022,10 @@
       <c r="D6" s="32"/>
       <c r="E6" s="32"/>
       <c r="F6" s="32"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="41"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="42"/>
+      <c r="J6" s="42"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>